<commit_message>
chore(saidas): regeração com os erros corrigidos
</commit_message>
<xml_diff>
--- a/apresentacoes_multiversao/Fatorial_Multiversao_numeros.xlsx
+++ b/apresentacoes_multiversao/Fatorial_Multiversao_numeros.xlsx
@@ -31673,10 +31673,10 @@
         <v>2119</v>
       </c>
       <c r="C5" t="s">
-        <v>485</v>
+        <v>1579</v>
       </c>
       <c r="D5" t="s">
-        <v>2121</v>
+        <v>25</v>
       </c>
     </row>
   </sheetData>

</xml_diff>